<commit_message>
bad results for PIRNN
</commit_message>
<xml_diff>
--- a/PIRNN/01-Pwm-XYTheta/Ts-03/Resumo_Estatisticas.xlsx
+++ b/PIRNN/01-Pwm-XYTheta/Ts-03/Resumo_Estatisticas.xlsx
@@ -473,16 +473,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.843941144619933</v>
+        <v>-0.496131398374039</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1752734173059962</v>
+        <v>5.243141042414061</v>
       </c>
       <c r="E2" t="n">
-        <v>0.03562302874322418</v>
+        <v>0.3415168698893713</v>
       </c>
       <c r="F2" t="n">
-        <v>0.04000907200945757</v>
+        <v>1.19683412776428</v>
       </c>
     </row>
     <row r="3">
@@ -497,16 +497,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.2176442196497463</v>
+        <v>-0.9072439373140553</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6205667533172329</v>
+        <v>5.953265093250761</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1786143836979396</v>
+        <v>0.4354300293818636</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1416774196230337</v>
+        <v>1.359149893601341</v>
       </c>
     </row>
     <row r="4">
@@ -521,16 +521,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.3161975655246781</v>
+        <v>-3.229632190769391</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7347460319148847</v>
+        <v>3.01749466208609</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2237946518833091</v>
+        <v>1.384272731427129</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2404674568922855</v>
+        <v>0.9875647312947247</v>
       </c>
     </row>
     <row r="5">
@@ -545,16 +545,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.6425799680265676</v>
+        <v>-0.5260169025107517</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2564167366297484</v>
+        <v>4.797937217523256</v>
       </c>
       <c r="E5" t="n">
-        <v>0.08210619847429758</v>
+        <v>0.3505551884735829</v>
       </c>
       <c r="F5" t="n">
-        <v>0.05890381508168727</v>
+        <v>1.102177690696603</v>
       </c>
     </row>
     <row r="6">
@@ -569,16 +569,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.2085114176853708</v>
+        <v>-0.8927124169980418</v>
       </c>
       <c r="D6" t="n">
-        <v>1.014816941636615</v>
+        <v>5.79285496884958</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2866118091121763</v>
+        <v>0.4488776208700402</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2406750282237544</v>
+        <v>1.37383943440631</v>
       </c>
     </row>
     <row r="7">
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-1.186453393151072</v>
+        <v>-2.165604567843752</v>
       </c>
       <c r="D7" t="n">
-        <v>1.129607485261155</v>
+        <v>5.308018472987801</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7187909635679512</v>
+        <v>1.040684409154611</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3713555730608405</v>
+        <v>1.744997503622419</v>
       </c>
     </row>
     <row r="8">
@@ -617,16 +617,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.7860197348817902</v>
+        <v>-0.1583296046334549</v>
       </c>
       <c r="D8" t="n">
-        <v>0.04086906732794032</v>
+        <v>0.2979030554452733</v>
       </c>
       <c r="E8" t="n">
-        <v>0.02307257808014477</v>
+        <v>0.1248977340535796</v>
       </c>
       <c r="F8" t="n">
-        <v>0.004406736978597897</v>
+        <v>0.03212161412772191</v>
       </c>
     </row>
     <row r="9">
@@ -641,16 +641,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-0.5603935544225919</v>
+        <v>-0.1890197459050597</v>
       </c>
       <c r="D9" t="n">
-        <v>0.05693998412736389</v>
+        <v>0.3604641072090072</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1314792910538985</v>
+        <v>0.1001872077704991</v>
       </c>
       <c r="F9" t="n">
-        <v>0.004797782408461892</v>
+        <v>0.03037282814447042</v>
       </c>
     </row>
     <row r="10">
@@ -665,16 +665,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-1.172373690997498</v>
+        <v>-1.123465290141928</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5769043928517587</v>
+        <v>0.6458770265804135</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2077291731205703</v>
+        <v>0.2030523987191495</v>
       </c>
       <c r="F10" t="n">
-        <v>0.05516540408924445</v>
+        <v>0.061760783250655</v>
       </c>
     </row>
     <row r="11">
@@ -689,16 +689,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6586399719819334</v>
+        <v>-0.281960809534035</v>
       </c>
       <c r="D11" t="n">
-        <v>0.07470974179339594</v>
+        <v>0.3250238342746891</v>
       </c>
       <c r="E11" t="n">
-        <v>0.03576108939168354</v>
+        <v>0.1342990137789516</v>
       </c>
       <c r="F11" t="n">
-        <v>0.007826639135856376</v>
+        <v>0.03404969954862358</v>
       </c>
     </row>
     <row r="12">
@@ -713,16 +713,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.5924881659693975</v>
+        <v>-0.2554128808622875</v>
       </c>
       <c r="D12" t="n">
-        <v>0.05335636509734738</v>
+        <v>0.3905113876597426</v>
       </c>
       <c r="E12" t="n">
-        <v>0.131050962590082</v>
+        <v>0.1033119554673993</v>
       </c>
       <c r="F12" t="n">
-        <v>0.004390866541892774</v>
+        <v>0.03213643551570442</v>
       </c>
     </row>
     <row r="13">
@@ -737,16 +737,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-2.17394035152952</v>
+        <v>-1.558278379805186</v>
       </c>
       <c r="D13" t="n">
-        <v>1.237224146862464</v>
+        <v>1.276953346240735</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2920163962520753</v>
+        <v>0.235372801735326</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1138300335570956</v>
+        <v>0.1174852936891369</v>
       </c>
     </row>
     <row r="14">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-2.006470769213967</v>
+        <v>-1.191342675507998</v>
       </c>
       <c r="D14" t="n">
-        <v>0.07933865081827969</v>
+        <v>1.702484246644834</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2519301385680117</v>
+        <v>0.1836256881469908</v>
       </c>
       <c r="F14" t="n">
-        <v>0.006648259314250399</v>
+        <v>0.142661321227223</v>
       </c>
     </row>
     <row r="15">
@@ -785,16 +785,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-2.792181806346063</v>
+        <v>-1.080337312208391</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1099442119554615</v>
+        <v>1.59475594835804</v>
       </c>
       <c r="E15" t="n">
-        <v>0.4083348334858467</v>
+        <v>0.2240067152248467</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0118385810001086</v>
+        <v>0.1717202491540876</v>
       </c>
     </row>
     <row r="16">
@@ -809,16 +809,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-2.391583606228379</v>
+        <v>-3.523955766968584</v>
       </c>
       <c r="D16" t="n">
-        <v>0.3787724212385292</v>
+        <v>2.332468161950916</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2525032585741352</v>
+        <v>0.336808318894763</v>
       </c>
       <c r="F16" t="n">
-        <v>0.02819959102441287</v>
+        <v>0.1736521577505737</v>
       </c>
     </row>
     <row r="17">
@@ -833,16 +833,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-2.246246705525828</v>
+        <v>-1.606009049675801</v>
       </c>
       <c r="D17" t="n">
-        <v>0.09841107644359808</v>
+        <v>1.743269293944142</v>
       </c>
       <c r="E17" t="n">
-        <v>0.2660263037503563</v>
+        <v>0.2135595405750089</v>
       </c>
       <c r="F17" t="n">
-        <v>0.008064678161958589</v>
+        <v>0.1428589780068285</v>
       </c>
     </row>
     <row r="18">
@@ -857,16 +857,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-2.742484839921008</v>
+        <v>-1.09452690972556</v>
       </c>
       <c r="D18" t="n">
-        <v>0.1260952960034312</v>
+        <v>1.597479516104396</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3972373459269541</v>
+        <v>0.2223186856274689</v>
       </c>
       <c r="F18" t="n">
-        <v>0.01338409181620998</v>
+        <v>0.1695607464807738</v>
       </c>
     </row>
     <row r="19">
@@ -881,16 +881,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-2.5717577714129</v>
+        <v>-3.738360657505509</v>
       </c>
       <c r="D19" t="n">
-        <v>0.4646610673453816</v>
+        <v>3.202578873261376</v>
       </c>
       <c r="E19" t="n">
-        <v>0.2743368906737135</v>
+        <v>0.3639404497345023</v>
       </c>
       <c r="F19" t="n">
-        <v>0.03568933858082865</v>
+        <v>0.2459812748948828</v>
       </c>
     </row>
   </sheetData>
@@ -951,16 +951,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.843941144619933</v>
+        <v>0.9117553928854594</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1752734173059962</v>
+        <v>0.01273121411535353</v>
       </c>
       <c r="E2" t="n">
-        <v>0.03562302874322418</v>
+        <v>0.02014329893692988</v>
       </c>
       <c r="F2" t="n">
-        <v>0.04000907200945757</v>
+        <v>0.002906111321032459</v>
       </c>
     </row>
     <row r="3">
@@ -975,16 +975,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.2176442196497463</v>
+        <v>0.8006499992806149</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6205667533172329</v>
+        <v>0.02527420522528277</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1786143836979396</v>
+        <v>0.04551225722744195</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1416774196230337</v>
+        <v>0.005770183723507606</v>
       </c>
     </row>
     <row r="4">
@@ -999,16 +999,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.3161975655246781</v>
+        <v>-3.72659970756937</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7347460319148847</v>
+        <v>3.124574051196847</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2237946518833091</v>
+        <v>1.546920108523557</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2404674568922855</v>
+        <v>1.022609641054817</v>
       </c>
     </row>
     <row r="5">
@@ -1023,16 +1023,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.6425799680265676</v>
+        <v>0.8292860733343492</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2564167366297484</v>
+        <v>0.0533305598409891</v>
       </c>
       <c r="E5" t="n">
-        <v>0.08210619847429758</v>
+        <v>0.03921624500939691</v>
       </c>
       <c r="F5" t="n">
-        <v>0.05890381508168727</v>
+        <v>0.01225104677785697</v>
       </c>
     </row>
     <row r="6">
@@ -1047,16 +1047,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.2085114176853708</v>
+        <v>0.841244155242995</v>
       </c>
       <c r="D6" t="n">
-        <v>1.014816941636615</v>
+        <v>0.05286711002240125</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2866118091121763</v>
+        <v>0.03765069920488169</v>
       </c>
       <c r="F6" t="n">
-        <v>0.2406750282237544</v>
+        <v>0.0125380181141141</v>
       </c>
     </row>
     <row r="7">
@@ -1071,16 +1071,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-1.186453393151072</v>
+        <v>0.6205177952636316</v>
       </c>
       <c r="D7" t="n">
-        <v>1.129607485261155</v>
+        <v>0.07374690563439308</v>
       </c>
       <c r="E7" t="n">
-        <v>0.7187909635679512</v>
+        <v>0.124753804702069</v>
       </c>
       <c r="F7" t="n">
-        <v>0.3713555730608405</v>
+        <v>0.0242441067013577</v>
       </c>
     </row>
     <row r="8">
@@ -1095,16 +1095,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.7860197348817902</v>
+        <v>-0.008507191627150057</v>
       </c>
       <c r="D8" t="n">
-        <v>0.04086906732794032</v>
+        <v>0.5729528074284169</v>
       </c>
       <c r="E8" t="n">
-        <v>0.02307257808014477</v>
+        <v>0.1087430231491229</v>
       </c>
       <c r="F8" t="n">
-        <v>0.004406736978597897</v>
+        <v>0.0617790541493507</v>
       </c>
     </row>
     <row r="9">
@@ -1119,16 +1119,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-0.5603935544225919</v>
+        <v>-0.4755456576377082</v>
       </c>
       <c r="D9" t="n">
-        <v>0.05693998412736389</v>
+        <v>0.7065958594413817</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1314792910538985</v>
+        <v>0.1243299784429406</v>
       </c>
       <c r="F9" t="n">
-        <v>0.004797782408461892</v>
+        <v>0.05953800718905861</v>
       </c>
     </row>
     <row r="10">
@@ -1143,16 +1143,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-1.172373690997498</v>
+        <v>-1.833977281990016</v>
       </c>
       <c r="D10" t="n">
-        <v>0.5769043928517587</v>
+        <v>0.929933007981094</v>
       </c>
       <c r="E10" t="n">
-        <v>0.2077291731205703</v>
+        <v>0.2709937796935625</v>
       </c>
       <c r="F10" t="n">
-        <v>0.05516540408924445</v>
+        <v>0.08892310545186942</v>
       </c>
     </row>
     <row r="11">
@@ -1167,16 +1167,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.6586399719819334</v>
+        <v>-0.2374804815798528</v>
       </c>
       <c r="D11" t="n">
-        <v>0.07470974179339594</v>
+        <v>0.6755965468563936</v>
       </c>
       <c r="E11" t="n">
-        <v>0.03576108939168354</v>
+        <v>0.129639226886572</v>
       </c>
       <c r="F11" t="n">
-        <v>0.007826639135856376</v>
+        <v>0.07077591551980283</v>
       </c>
     </row>
     <row r="12">
@@ -1191,16 +1191,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.5924881659693975</v>
+        <v>-0.5444172149178019</v>
       </c>
       <c r="D12" t="n">
-        <v>0.05335636509734738</v>
+        <v>0.7771529314495381</v>
       </c>
       <c r="E12" t="n">
-        <v>0.131050962590082</v>
+        <v>0.1270950497346182</v>
       </c>
       <c r="F12" t="n">
-        <v>0.004390866541892774</v>
+        <v>0.06395440915830525</v>
       </c>
     </row>
     <row r="13">
@@ -1215,16 +1215,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-2.17394035152952</v>
+        <v>-3.035108145284216</v>
       </c>
       <c r="D13" t="n">
-        <v>1.237224146862464</v>
+        <v>1.982258184255975</v>
       </c>
       <c r="E13" t="n">
-        <v>0.2920163962520753</v>
+        <v>0.3712476003228799</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1138300335570956</v>
+        <v>0.1823764240335089</v>
       </c>
     </row>
     <row r="14">
@@ -1239,16 +1239,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-2.006470769213967</v>
+        <v>-2.408856728638173</v>
       </c>
       <c r="D14" t="n">
-        <v>0.07933865081827969</v>
+        <v>3.451825852232595</v>
       </c>
       <c r="E14" t="n">
-        <v>0.2519301385680117</v>
+        <v>0.2856484609124748</v>
       </c>
       <c r="F14" t="n">
-        <v>0.006648259314250399</v>
+        <v>0.2892491003639333</v>
       </c>
     </row>
     <row r="15">
@@ -1263,16 +1263,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-2.792181806346063</v>
+        <v>-2.229663313340679</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1099442119554615</v>
+        <v>3.230261982649708</v>
       </c>
       <c r="E15" t="n">
-        <v>0.4083348334858467</v>
+        <v>0.3477639255220787</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0118385810001086</v>
+        <v>0.3478283890802886</v>
       </c>
     </row>
     <row r="16">
@@ -1287,16 +1287,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-2.391583606228379</v>
+        <v>-4.238009299691236</v>
       </c>
       <c r="D16" t="n">
-        <v>0.3787724212385292</v>
+        <v>0.4549486946345115</v>
       </c>
       <c r="E16" t="n">
-        <v>0.2525032585741352</v>
+        <v>0.3899695747392996</v>
       </c>
       <c r="F16" t="n">
-        <v>0.02819959102441287</v>
+        <v>0.0338709114138606</v>
       </c>
     </row>
     <row r="17">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>-2.246246705525828</v>
+        <v>-2.905269145502048</v>
       </c>
       <c r="D17" t="n">
-        <v>0.09841107644359808</v>
+        <v>3.491117539618979</v>
       </c>
       <c r="E17" t="n">
-        <v>0.2660263037503563</v>
+        <v>0.3200324590733593</v>
       </c>
       <c r="F17" t="n">
-        <v>0.008064678161958589</v>
+        <v>0.2860931960106339</v>
       </c>
     </row>
     <row r="18">
@@ -1335,16 +1335,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>-2.742484839921008</v>
+        <v>-2.222707312830275</v>
       </c>
       <c r="D18" t="n">
-        <v>0.1260952960034312</v>
+        <v>3.245733923960367</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3972373459269541</v>
+        <v>0.342066769647918</v>
       </c>
       <c r="F18" t="n">
-        <v>0.01338409181620998</v>
+        <v>0.3445108757117393</v>
       </c>
     </row>
     <row r="19">
@@ -1359,16 +1359,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>-2.5717577714129</v>
+        <v>-4.475771574076486</v>
       </c>
       <c r="D19" t="n">
-        <v>0.4646610673453816</v>
+        <v>0.3732028592601934</v>
       </c>
       <c r="E19" t="n">
-        <v>0.2743368906737135</v>
+        <v>0.4205789540642374</v>
       </c>
       <c r="F19" t="n">
-        <v>0.03568933858082865</v>
+        <v>0.02866468516410076</v>
       </c>
     </row>
   </sheetData>

</xml_diff>